<commit_message>
fix: ajustar normalizacao de produtos do mapa
- padroniza saidas de cogumelos com BANDEJA 200g
- corrige correspondencia de QUIABO BANDEJA 300G
- adiciona BATATA CALABRESA como BATATA BOLINHA
- ajusta saidas de ovos C/20 e C/30
- evita interpretar C/20 como quantidade
- padroniza PERA WILLIAMS como PÊRA WILLIANS
</commit_message>
<xml_diff>
--- a/template/mapa/MAPA.xlsx
+++ b/template/mapa/MAPA.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EBBE041-3176-4546-9DDB-061A8AFF077C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09484A00-1C1C-47DE-AF64-796FF43629AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan2" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="123">
   <si>
     <t>FEIRA NOVA</t>
   </si>
@@ -251,9 +251,6 @@
     <t>OVOS C/12</t>
   </si>
   <si>
-    <t>OVOS  BRANCOS C/30</t>
-  </si>
-  <si>
     <t>OVOS BRANCO C/ 20</t>
   </si>
   <si>
@@ -378,6 +375,15 @@
   </si>
   <si>
     <t>UVA THOMPSON</t>
+  </si>
+  <si>
+    <t>ROMA</t>
+  </si>
+  <si>
+    <t>COGUMELO PARIS BANDEJA 200g</t>
+  </si>
+  <si>
+    <t>OVOS BRANCOS C/30</t>
   </si>
 </sst>
 </file>
@@ -596,6 +602,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -603,15 +618,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -987,7 +993,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
@@ -1045,33 +1051,33 @@
       <c r="A5" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="10"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="13"/>
       <c r="E5" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="G5" s="9"/>
-      <c r="H5" s="10"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="13"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="7"/>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="12"/>
-      <c r="D6" s="13"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="10"/>
       <c r="E6" s="7"/>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="G6" s="12"/>
-      <c r="H6" s="13"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="10"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="7"/>
@@ -1141,7 +1147,7 @@
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
@@ -1155,7 +1161,7 @@
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
@@ -1197,7 +1203,7 @@
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
@@ -1211,7 +1217,7 @@
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
@@ -1239,7 +1245,7 @@
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
@@ -1281,7 +1287,7 @@
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
@@ -1295,7 +1301,7 @@
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -1323,7 +1329,7 @@
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
@@ -1337,7 +1343,7 @@
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
@@ -1351,7 +1357,7 @@
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
@@ -1365,7 +1371,7 @@
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
@@ -1393,7 +1399,7 @@
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
@@ -1407,7 +1413,7 @@
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
@@ -1435,7 +1441,7 @@
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
@@ -1463,7 +1469,7 @@
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
       <c r="E34" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
@@ -1491,7 +1497,7 @@
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
       <c r="E36" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
@@ -1505,7 +1511,7 @@
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
       <c r="E37" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
@@ -1547,7 +1553,7 @@
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
       <c r="E40" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
@@ -1601,7 +1607,7 @@
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
       <c r="E44" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
@@ -1615,7 +1621,7 @@
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
       <c r="E45" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
@@ -1629,7 +1635,7 @@
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
       <c r="E46" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
@@ -1699,7 +1705,7 @@
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
       <c r="E51" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
@@ -1711,7 +1717,7 @@
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
       <c r="E52" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F52" s="3"/>
       <c r="G52" s="3"/>
@@ -1725,7 +1731,7 @@
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
       <c r="E53" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
@@ -1753,7 +1759,7 @@
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
       <c r="E55" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
@@ -1761,13 +1767,13 @@
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>78</v>
+        <v>122</v>
       </c>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
       <c r="D56" s="3"/>
       <c r="E56" s="1" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="3"/>
@@ -1775,13 +1781,13 @@
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
       <c r="D57" s="3"/>
       <c r="E57" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
@@ -1789,13 +1795,13 @@
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
       <c r="E58" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F58" s="3"/>
       <c r="G58" s="3"/>
@@ -1803,13 +1809,13 @@
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
       <c r="E59" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F59" s="3"/>
       <c r="G59" s="3"/>
@@ -1817,13 +1823,13 @@
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
       <c r="E60" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F60" s="3"/>
       <c r="G60" s="3"/>
@@ -1831,13 +1837,13 @@
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
       <c r="E61" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F61" s="3"/>
       <c r="G61" s="3"/>
@@ -1845,13 +1851,13 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
       <c r="D62" s="3"/>
       <c r="E62" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F62" s="3"/>
       <c r="G62" s="3"/>
@@ -1859,13 +1865,13 @@
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
-        <v>85</v>
+        <v>121</v>
       </c>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
       <c r="D63" s="3"/>
       <c r="E63" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F63" s="3"/>
       <c r="G63" s="3"/>
@@ -1873,13 +1879,13 @@
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
       <c r="D64" s="3"/>
       <c r="E64" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F64" s="3"/>
       <c r="G64" s="3"/>
@@ -1887,17 +1893,31 @@
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
-        <v>48</v>
+        <v>85</v>
       </c>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
       <c r="D65" s="3"/>
       <c r="E65" s="1" t="s">
-        <v>49</v>
+        <v>119</v>
       </c>
       <c r="F65" s="3"/>
       <c r="G65" s="3"/>
       <c r="H65" s="3"/>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A66" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B66" s="3"/>
+      <c r="C66" s="3"/>
+      <c r="D66" s="3"/>
+      <c r="E66" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F66" s="3"/>
+      <c r="G66" s="3"/>
+      <c r="H66" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
Organiza produtos de frutas em ordem alfabética
</commit_message>
<xml_diff>
--- a/template/mapa/MAPA.xlsx
+++ b/template/mapa/MAPA.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09484A00-1C1C-47DE-AF64-796FF43629AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4B6E5DF-0764-425D-A307-97019B78604C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan2" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="9">
   <si>
     <t>FEIRA NOVA</t>
   </si>
@@ -35,138 +35,6 @@
     <t>QUEIM</t>
   </si>
   <si>
-    <t>ABÓBORA SERGIPANA</t>
-  </si>
-  <si>
-    <t>ABACATE</t>
-  </si>
-  <si>
-    <t>ABOBRINHA</t>
-  </si>
-  <si>
-    <t>ABACAXI (Unid.)</t>
-  </si>
-  <si>
-    <t>AIPIM</t>
-  </si>
-  <si>
-    <t>BANANA DA TERRA</t>
-  </si>
-  <si>
-    <t>BATATA BAROA</t>
-  </si>
-  <si>
-    <t>BANANA D'ÀGUA</t>
-  </si>
-  <si>
-    <t>BATATA DOCE</t>
-  </si>
-  <si>
-    <t>BANANA PRATA</t>
-  </si>
-  <si>
-    <t>BERINJELA</t>
-  </si>
-  <si>
-    <t>CAQUI RAMA FORTE KG</t>
-  </si>
-  <si>
-    <t>BETERRABA</t>
-  </si>
-  <si>
-    <t>CÔCO SECO UN</t>
-  </si>
-  <si>
-    <t>CENOURA</t>
-  </si>
-  <si>
-    <t>GOIABA granel</t>
-  </si>
-  <si>
-    <t>CHUCHU</t>
-  </si>
-  <si>
-    <t>LARANJA PERA</t>
-  </si>
-  <si>
-    <t>INHAME</t>
-  </si>
-  <si>
-    <t>LIMÃO</t>
-  </si>
-  <si>
-    <t>JILO</t>
-  </si>
-  <si>
-    <t>MACA 850G</t>
-  </si>
-  <si>
-    <t>PEPINO</t>
-  </si>
-  <si>
-    <t>MACA GALA</t>
-  </si>
-  <si>
-    <t>PIMENTÃO</t>
-  </si>
-  <si>
-    <t>MAMÃO FORMOSA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOMATE </t>
-  </si>
-  <si>
-    <t>MAMÃO HAVAI</t>
-  </si>
-  <si>
-    <t>TOMATE SWEET 180</t>
-  </si>
-  <si>
-    <t>MANGA palmer</t>
-  </si>
-  <si>
-    <t>MANGA TOMMY</t>
-  </si>
-  <si>
-    <t>BATATA ASTERIX</t>
-  </si>
-  <si>
-    <t>MARACUJÁ</t>
-  </si>
-  <si>
-    <t>BATATA INGLESA</t>
-  </si>
-  <si>
-    <t>MELAO ORANGE</t>
-  </si>
-  <si>
-    <t>CEBOLA ROXA</t>
-  </si>
-  <si>
-    <t>MELAO VERDE</t>
-  </si>
-  <si>
-    <t>MILHO VERDE BDJ 3</t>
-  </si>
-  <si>
-    <t>ALHO</t>
-  </si>
-  <si>
-    <t>MORANGO</t>
-  </si>
-  <si>
-    <t>ALHO DESCASCADO</t>
-  </si>
-  <si>
-    <t>PINHA</t>
-  </si>
-  <si>
-    <t>QUIABO BANDEJA 300G</t>
-  </si>
-  <si>
-    <t>UVA VITORIA</t>
-  </si>
-  <si>
     <t>Descrição dos Produtos</t>
   </si>
   <si>
@@ -174,216 +42,6 @@
   </si>
   <si>
     <t>DATA 28/04/2026</t>
-  </si>
-  <si>
-    <t>ABOBORA BAIANA</t>
-  </si>
-  <si>
-    <t>ABOBORA JAPONESA</t>
-  </si>
-  <si>
-    <t>ABOBORA MORANGA</t>
-  </si>
-  <si>
-    <t>ABOBORA PESCOCO</t>
-  </si>
-  <si>
-    <t>COUVE FLOR</t>
-  </si>
-  <si>
-    <t>ERVILHA</t>
-  </si>
-  <si>
-    <t>GENGIBRE</t>
-  </si>
-  <si>
-    <t>MAXIXE</t>
-  </si>
-  <si>
-    <t>NABO</t>
-  </si>
-  <si>
-    <t>PEPINO JAPONES</t>
-  </si>
-  <si>
-    <t>PIMENTÃO AMARELO</t>
-  </si>
-  <si>
-    <t>PIMENTÃO VERMELHO</t>
-  </si>
-  <si>
-    <t>REPOLHO</t>
-  </si>
-  <si>
-    <t>REPOLHO ROXO</t>
-  </si>
-  <si>
-    <t>TOMATE ITALIANO</t>
-  </si>
-  <si>
-    <t>VAGEM MANT</t>
-  </si>
-  <si>
-    <t>PIMENTA DEDO MOCA BANDEJA 200g</t>
-  </si>
-  <si>
-    <t>PIMENTA MALAGUETA BANDEJA 150g</t>
-  </si>
-  <si>
-    <t>BATATA BOLINHA</t>
-  </si>
-  <si>
-    <t>BATATA SUJA</t>
-  </si>
-  <si>
-    <t>CARA</t>
-  </si>
-  <si>
-    <t>CEBOLA</t>
-  </si>
-  <si>
-    <t>CEBOLA PIRULITO</t>
-  </si>
-  <si>
-    <t>CEBOLA ROXA PCT</t>
-  </si>
-  <si>
-    <t>OVOS C/12</t>
-  </si>
-  <si>
-    <t>OVOS BRANCO C/ 20</t>
-  </si>
-  <si>
-    <t>OVOS CODORNA C/ 30</t>
-  </si>
-  <si>
-    <t>OVOS VERMELHOS C/12</t>
-  </si>
-  <si>
-    <t>OVOS VERMELHOS C/20</t>
-  </si>
-  <si>
-    <t>OVOS VERMELHOS C/30</t>
-  </si>
-  <si>
-    <t>COGUMELO PORTOBELLO BANDEJA 200g</t>
-  </si>
-  <si>
-    <t>COGUMELO SHIMEJI BANDEJA 200g</t>
-  </si>
-  <si>
-    <t>COGUMELO SHITAKE BANDEJA 200g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMEIXA </t>
-  </si>
-  <si>
-    <t>AMEIXA RUBIMEL</t>
-  </si>
-  <si>
-    <t>BANANA MAÇÃ</t>
-  </si>
-  <si>
-    <t>BANANA OURO</t>
-  </si>
-  <si>
-    <t>CAJU</t>
-  </si>
-  <si>
-    <t>CÔCO VERDE</t>
-  </si>
-  <si>
-    <t>FIGO</t>
-  </si>
-  <si>
-    <t>KIWI KG</t>
-  </si>
-  <si>
-    <t>LARANJA  SELETA</t>
-  </si>
-  <si>
-    <t>LARANJA BAHIA</t>
-  </si>
-  <si>
-    <t>LARANJA LIMA</t>
-  </si>
-  <si>
-    <t>COGUMELO</t>
-  </si>
-  <si>
-    <t>LIMA DA PERSIA</t>
-  </si>
-  <si>
-    <t>LIMÃO SICILIANO</t>
-  </si>
-  <si>
-    <t>MACA FUJI</t>
-  </si>
-  <si>
-    <t>MACA RED IMPORT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MACA VERDE GRAN </t>
-  </si>
-  <si>
-    <t>MELAO CANT</t>
-  </si>
-  <si>
-    <t>MELANCIA</t>
-  </si>
-  <si>
-    <t>MELANCIA BABY</t>
-  </si>
-  <si>
-    <t>MELÃO AMARELO</t>
-  </si>
-  <si>
-    <t>PÊRA PORTUGUESA</t>
-  </si>
-  <si>
-    <t>PÊRA WILLIANS</t>
-  </si>
-  <si>
-    <t>PESSEGO</t>
-  </si>
-  <si>
-    <t>PITAYA</t>
-  </si>
-  <si>
-    <t>SERIGUELA</t>
-  </si>
-  <si>
-    <t>TANGERINA IMP</t>
-  </si>
-  <si>
-    <t>TANGERINA PONKAN</t>
-  </si>
-  <si>
-    <t>TANGERINA MORCOTE</t>
-  </si>
-  <si>
-    <t>UVA CRIMSON</t>
-  </si>
-  <si>
-    <t>UVA ITÁLIA</t>
-  </si>
-  <si>
-    <t>UVA RED GLOB</t>
-  </si>
-  <si>
-    <t>UVA ROSADA</t>
-  </si>
-  <si>
-    <t>UVA THOMPSON</t>
-  </si>
-  <si>
-    <t>ROMA</t>
-  </si>
-  <si>
-    <t>COGUMELO PARIS BANDEJA 200g</t>
-  </si>
-  <si>
-    <t>OVOS BRANCOS C/30</t>
   </si>
 </sst>
 </file>
@@ -590,6 +248,36 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -602,6 +290,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -610,45 +307,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1002,85 +660,85 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="16"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="6"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="23"/>
-      <c r="B2" s="23"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="19"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="9"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="23"/>
-      <c r="B3" s="23"/>
-      <c r="C3" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="22"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="12"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="4"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="6"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="16"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B5" s="11" t="s">
+      <c r="A5" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="12"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="F5" s="11" t="s">
+      <c r="C5" s="19"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="G5" s="12"/>
-      <c r="H5" s="13"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="7"/>
-      <c r="B6" s="8" t="s">
+      <c r="A6" s="17"/>
+      <c r="B6" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="8" t="s">
+      <c r="C6" s="22"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="G6" s="9"/>
-      <c r="H6" s="10"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="7"/>
+      <c r="A7" s="17"/>
       <c r="B7" s="2" t="s">
         <v>3</v>
       </c>
@@ -1090,7 +748,7 @@
       <c r="D7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="7"/>
+      <c r="E7" s="17"/>
       <c r="F7" s="2" t="s">
         <v>3</v>
       </c>
@@ -1102,473 +760,341 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="6"/>
+      <c r="A8" s="15"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="16"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>53</v>
-      </c>
+      <c r="A9" s="1"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
-      <c r="E9" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="E9" s="1"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>54</v>
-      </c>
+      <c r="A10" s="1"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
-      <c r="E10" s="1" t="s">
-        <v>9</v>
-      </c>
+      <c r="E10" s="1"/>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>55</v>
-      </c>
+      <c r="A11" s="1"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
-      <c r="E11" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="E11" s="1"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>56</v>
-      </c>
+      <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
-      <c r="E12" s="1" t="s">
-        <v>87</v>
-      </c>
+      <c r="E12" s="1"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>6</v>
-      </c>
+      <c r="A13" s="1"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
-      <c r="E13" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="E13" s="1"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="A14" s="1"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
-      <c r="E14" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="E14" s="1"/>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="A15" s="1"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
-      <c r="E15" s="1" t="s">
-        <v>88</v>
-      </c>
+      <c r="E15" s="1"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="A16" s="1"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
-      <c r="E16" s="1" t="s">
-        <v>89</v>
-      </c>
+      <c r="E16" s="1"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="A17" s="1"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
-      <c r="E17" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="E17" s="1"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>16</v>
-      </c>
+      <c r="A18" s="1"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
-      <c r="E18" s="1" t="s">
-        <v>90</v>
-      </c>
+      <c r="E18" s="1"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>18</v>
-      </c>
+      <c r="A19" s="1"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
-      <c r="E19" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="E19" s="1"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>20</v>
-      </c>
+      <c r="A20" s="1"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
-      <c r="E20" s="1" t="s">
-        <v>19</v>
-      </c>
+      <c r="E20" s="1"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>22</v>
-      </c>
+      <c r="A21" s="1"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
-      <c r="E21" s="1" t="s">
-        <v>91</v>
-      </c>
+      <c r="E21" s="1"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>57</v>
-      </c>
+      <c r="A22" s="1"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
-      <c r="E22" s="1" t="s">
-        <v>92</v>
-      </c>
+      <c r="E22" s="1"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>58</v>
-      </c>
+      <c r="A23" s="1"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
-      <c r="E23" s="1" t="s">
-        <v>21</v>
-      </c>
+      <c r="E23" s="1"/>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>59</v>
-      </c>
+      <c r="A24" s="1"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
-      <c r="E24" s="1" t="s">
-        <v>93</v>
-      </c>
+      <c r="E24" s="1"/>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="A25" s="1"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
-      <c r="E25" s="1" t="s">
-        <v>94</v>
-      </c>
+      <c r="E25" s="1"/>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="A26" s="1"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
-      <c r="E26" s="1" t="s">
-        <v>95</v>
-      </c>
+      <c r="E26" s="1"/>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
-        <v>60</v>
-      </c>
+      <c r="A27" s="1"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
-      <c r="E27" s="1" t="s">
-        <v>96</v>
-      </c>
+      <c r="E27" s="1"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
-        <v>61</v>
-      </c>
+      <c r="A28" s="1"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
-      <c r="E28" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="E28" s="1"/>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
-        <v>28</v>
-      </c>
+      <c r="A29" s="1"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
-      <c r="E29" s="1" t="s">
-        <v>97</v>
-      </c>
+      <c r="E29" s="1"/>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
-        <v>62</v>
-      </c>
+      <c r="A30" s="1"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
-      <c r="E30" s="1" t="s">
-        <v>98</v>
-      </c>
+      <c r="E30" s="1"/>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
-        <v>30</v>
-      </c>
+      <c r="A31" s="1"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
-      <c r="E31" s="1" t="s">
-        <v>25</v>
-      </c>
+      <c r="E31" s="1"/>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
-        <v>63</v>
-      </c>
+      <c r="A32" s="1"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
-      <c r="E32" s="1" t="s">
-        <v>99</v>
-      </c>
+      <c r="E32" s="1"/>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
-        <v>64</v>
-      </c>
+      <c r="A33" s="1"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
-      <c r="E33" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="E33" s="1"/>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
-        <v>65</v>
-      </c>
+      <c r="A34" s="1"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
-      <c r="E34" s="1" t="s">
-        <v>100</v>
-      </c>
+      <c r="E34" s="1"/>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
-        <v>66</v>
-      </c>
+      <c r="A35" s="1"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
-      <c r="E35" s="1" t="s">
-        <v>29</v>
-      </c>
+      <c r="E35" s="1"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="A36" s="1"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
-      <c r="E36" s="1" t="s">
-        <v>101</v>
-      </c>
+      <c r="E36" s="1"/>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" s="1" t="s">
-        <v>67</v>
-      </c>
+      <c r="A37" s="1"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
-      <c r="E37" s="1" t="s">
-        <v>102</v>
-      </c>
+      <c r="E37" s="1"/>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A38" s="1" t="s">
-        <v>34</v>
-      </c>
+      <c r="A38" s="1"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
-      <c r="E38" s="1" t="s">
-        <v>31</v>
-      </c>
+      <c r="E38" s="1"/>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A39" s="1" t="s">
-        <v>68</v>
-      </c>
+      <c r="A39" s="1"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
-      <c r="E39" s="1" t="s">
-        <v>33</v>
-      </c>
+      <c r="E39" s="1"/>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A40" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="A40" s="1"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
-      <c r="E40" s="1" t="s">
-        <v>103</v>
-      </c>
+      <c r="E40" s="1"/>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A41" s="1" t="s">
-        <v>70</v>
-      </c>
+      <c r="A41" s="1"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
-      <c r="E41" s="1" t="s">
-        <v>35</v>
-      </c>
+      <c r="E41" s="1"/>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
@@ -1578,135 +1104,97 @@
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
-      <c r="E42" s="1" t="s">
-        <v>36</v>
-      </c>
+      <c r="E42" s="1"/>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A43" s="1" t="s">
-        <v>37</v>
-      </c>
+      <c r="A43" s="1"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
-      <c r="E43" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="E43" s="1"/>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A44" s="1" t="s">
-        <v>71</v>
-      </c>
+      <c r="A44" s="1"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
-      <c r="E44" s="1" t="s">
-        <v>104</v>
-      </c>
+      <c r="E44" s="1"/>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
       <c r="H44" s="3"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A45" s="1" t="s">
-        <v>39</v>
-      </c>
+      <c r="A45" s="1"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
-      <c r="E45" s="1" t="s">
-        <v>105</v>
-      </c>
+      <c r="E45" s="1"/>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
       <c r="H45" s="3"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A46" s="1" t="s">
-        <v>72</v>
-      </c>
+      <c r="A46" s="1"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
-      <c r="E46" s="1" t="s">
-        <v>106</v>
-      </c>
+      <c r="E46" s="1"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
       <c r="H46" s="3"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A47" s="1" t="s">
-        <v>73</v>
-      </c>
+      <c r="A47" s="1"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
-      <c r="E47" s="1" t="s">
-        <v>40</v>
-      </c>
+      <c r="E47" s="1"/>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
       <c r="H47" s="3"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A48" s="1" t="s">
-        <v>74</v>
-      </c>
+      <c r="A48" s="1"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
-      <c r="E48" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="E48" s="1"/>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
       <c r="H48" s="3"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A49" s="1" t="s">
-        <v>75</v>
-      </c>
+      <c r="A49" s="1"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
-      <c r="E49" s="1" t="s">
-        <v>43</v>
-      </c>
+      <c r="E49" s="1"/>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
       <c r="H49" s="3"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A50" s="1" t="s">
-        <v>41</v>
-      </c>
+      <c r="A50" s="1"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
-      <c r="E50" s="1" t="s">
-        <v>45</v>
-      </c>
+      <c r="E50" s="1"/>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
       <c r="H50" s="3"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A51" s="1" t="s">
-        <v>76</v>
-      </c>
+      <c r="A51" s="1"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
-      <c r="E51" s="1" t="s">
-        <v>107</v>
-      </c>
+      <c r="E51" s="1"/>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
       <c r="H51" s="3"/>
@@ -1716,211 +1204,158 @@
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
-      <c r="E52" s="1" t="s">
-        <v>108</v>
-      </c>
+      <c r="E52" s="1"/>
       <c r="F52" s="3"/>
       <c r="G52" s="3"/>
       <c r="H52" s="3"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A53" s="1" t="s">
-        <v>44</v>
-      </c>
+      <c r="A53" s="1"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
-      <c r="E53" s="1" t="s">
-        <v>109</v>
-      </c>
+      <c r="E53" s="1"/>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
       <c r="H53" s="3"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A54" s="1" t="s">
-        <v>46</v>
-      </c>
+      <c r="A54" s="1"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
-      <c r="E54" s="1" t="s">
-        <v>47</v>
-      </c>
+      <c r="E54" s="1"/>
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
       <c r="H54" s="3"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A55" s="1" t="s">
-        <v>77</v>
-      </c>
+      <c r="A55" s="1"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
-      <c r="E55" s="1" t="s">
-        <v>110</v>
-      </c>
+      <c r="E55" s="1"/>
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
       <c r="H55" s="3"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A56" s="1" t="s">
-        <v>122</v>
-      </c>
+      <c r="A56" s="1"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
       <c r="D56" s="3"/>
-      <c r="E56" s="1" t="s">
-        <v>120</v>
-      </c>
+      <c r="E56" s="1"/>
       <c r="F56" s="3"/>
       <c r="G56" s="3"/>
       <c r="H56" s="3"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A57" s="1" t="s">
-        <v>78</v>
-      </c>
+      <c r="A57" s="1"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
       <c r="D57" s="3"/>
-      <c r="E57" s="1" t="s">
-        <v>111</v>
-      </c>
+      <c r="E57" s="1"/>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
       <c r="H57" s="3"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A58" s="1" t="s">
-        <v>79</v>
-      </c>
+      <c r="A58" s="1"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
-      <c r="E58" s="1" t="s">
-        <v>112</v>
-      </c>
+      <c r="E58" s="1"/>
       <c r="F58" s="3"/>
       <c r="G58" s="3"/>
       <c r="H58" s="3"/>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A59" s="1" t="s">
-        <v>80</v>
-      </c>
+      <c r="A59" s="1"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
-      <c r="E59" s="1" t="s">
-        <v>113</v>
-      </c>
+      <c r="E59" s="1"/>
       <c r="F59" s="3"/>
       <c r="G59" s="3"/>
       <c r="H59" s="3"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A60" s="1" t="s">
-        <v>81</v>
-      </c>
+      <c r="A60" s="1"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
-      <c r="E60" s="1" t="s">
-        <v>114</v>
-      </c>
+      <c r="E60" s="1"/>
       <c r="F60" s="3"/>
       <c r="G60" s="3"/>
       <c r="H60" s="3"/>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A61" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="A61" s="1"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
-      <c r="E61" s="1" t="s">
-        <v>115</v>
-      </c>
+      <c r="E61" s="1"/>
       <c r="F61" s="3"/>
       <c r="G61" s="3"/>
       <c r="H61" s="3"/>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A62" s="1" t="s">
-        <v>83</v>
-      </c>
+      <c r="A62" s="1"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
       <c r="D62" s="3"/>
-      <c r="E62" s="1" t="s">
-        <v>116</v>
-      </c>
+      <c r="E62" s="1"/>
       <c r="F62" s="3"/>
       <c r="G62" s="3"/>
       <c r="H62" s="3"/>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A63" s="1" t="s">
-        <v>121</v>
-      </c>
+      <c r="A63" s="1"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
       <c r="D63" s="3"/>
-      <c r="E63" s="1" t="s">
-        <v>117</v>
-      </c>
+      <c r="E63" s="1"/>
       <c r="F63" s="3"/>
       <c r="G63" s="3"/>
       <c r="H63" s="3"/>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A64" s="1" t="s">
-        <v>84</v>
-      </c>
+      <c r="A64" s="1"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
       <c r="D64" s="3"/>
-      <c r="E64" s="1" t="s">
-        <v>118</v>
-      </c>
+      <c r="E64" s="1"/>
       <c r="F64" s="3"/>
       <c r="G64" s="3"/>
       <c r="H64" s="3"/>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A65" s="1" t="s">
-        <v>85</v>
-      </c>
+      <c r="A65" s="1"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
       <c r="D65" s="3"/>
-      <c r="E65" s="1" t="s">
-        <v>119</v>
-      </c>
+      <c r="E65" s="1"/>
       <c r="F65" s="3"/>
       <c r="G65" s="3"/>
       <c r="H65" s="3"/>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A66" s="1" t="s">
-        <v>48</v>
-      </c>
+      <c r="A66" s="1"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
       <c r="D66" s="3"/>
-      <c r="E66" s="1" t="s">
-        <v>49</v>
-      </c>
+      <c r="E66" s="1"/>
       <c r="F66" s="3"/>
       <c r="G66" s="3"/>
       <c r="H66" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B5:D5"/>
     <mergeCell ref="C1:H2"/>
     <mergeCell ref="C3:H3"/>
     <mergeCell ref="A1:B3"/>
@@ -1928,11 +1363,6 @@
     <mergeCell ref="E5:E7"/>
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="F6:H6"/>
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B5:D5"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Adiciona ervilha, maxixe e cajá às regras de fornecedores
</commit_message>
<xml_diff>
--- a/template/mapa/MAPA.xlsx
+++ b/template/mapa/MAPA.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4B6E5DF-0764-425D-A307-97019B78604C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3743D656-B4C6-41A0-934B-3868756F2419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -248,6 +248,36 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -277,36 +307,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -660,85 +660,85 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="4" t="s">
+      <c r="B1" s="23"/>
+      <c r="C1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="6"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="16"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="9"/>
+      <c r="A2" s="23"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="19"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="10" t="s">
+      <c r="A3" s="23"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="12"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="22"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="14"/>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="16"/>
+      <c r="A4" s="4"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="6"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="19"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="17" t="s">
+      <c r="C5" s="12"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="G5" s="19"/>
-      <c r="H5" s="20"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="13"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="17"/>
-      <c r="B6" s="21" t="s">
+      <c r="A6" s="7"/>
+      <c r="B6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="22"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="21" t="s">
+      <c r="C6" s="9"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="G6" s="22"/>
-      <c r="H6" s="23"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="10"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="17"/>
+      <c r="A7" s="7"/>
       <c r="B7" s="2" t="s">
         <v>3</v>
       </c>
@@ -748,7 +748,7 @@
       <c r="D7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="17"/>
+      <c r="E7" s="7"/>
       <c r="F7" s="2" t="s">
         <v>3</v>
       </c>
@@ -760,14 +760,14 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="15"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="16"/>
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="6"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1351,11 +1351,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B5:D5"/>
     <mergeCell ref="C1:H2"/>
     <mergeCell ref="C3:H3"/>
     <mergeCell ref="A1:B3"/>
@@ -1363,8 +1358,13 @@
     <mergeCell ref="E5:E7"/>
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="F6:H6"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B5:D5"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="76" fitToWidth="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>